<commit_message>
ive got maggots for brain
</commit_message>
<xml_diff>
--- a/scenario.xlsx
+++ b/scenario.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="80">
   <si>
     <t>AK-176</t>
   </si>
@@ -107,9 +107,6 @@
     <t>,-15-85</t>
   </si>
   <si>
-    <t>,-60-159</t>
-  </si>
-  <si>
     <t>0-11</t>
   </si>
   <si>
@@ -134,9 +131,6 @@
     <t>Điểm D3</t>
   </si>
   <si>
-    <t>Điểm kết thúc (D4)</t>
-  </si>
-  <si>
     <t>Tàu ta</t>
   </si>
   <si>
@@ -167,30 +161,15 @@
     <t>109.763434°W / 12.023436°N</t>
   </si>
   <si>
-    <t>Tên lửa YJ-83</t>
-  </si>
-  <si>
-    <t>1080 km/h</t>
-  </si>
-  <si>
     <t>10m</t>
   </si>
   <si>
     <t>Tàu khu trục D0</t>
   </si>
   <si>
-    <t>110.4359883°W / 11.921168°N</t>
-  </si>
-  <si>
-    <t>109.979486°W / 12.069443°N</t>
-  </si>
-  <si>
     <t>109.550867°W / 12.020027°N</t>
   </si>
   <si>
-    <t>78 km/h</t>
-  </si>
-  <si>
     <t>110.394166°W / 11.854674°N</t>
   </si>
   <si>
@@ -209,9 +188,6 @@
     <t>109.678059°W / 11.866610°N</t>
   </si>
   <si>
-    <t>150 km/h</t>
-  </si>
-  <si>
     <t>1000m</t>
   </si>
   <si>
@@ -243,13 +219,58 @@
   </si>
   <si>
     <t>109.636242°W / 11.440001°N</t>
+  </si>
+  <si>
+    <t>Mức Hiểm Họa (HH)</t>
+  </si>
+  <si>
+    <t>D4</t>
+  </si>
+  <si>
+    <t>Rất Cao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tên lửa YJ-83 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rất Cao </t>
+  </si>
+  <si>
+    <t>Trùng D2 Khu trục</t>
+  </si>
+  <si>
+    <t>109.530830°W / 11.985940°N</t>
+  </si>
+  <si>
+    <t>Cao</t>
+  </si>
+  <si>
+    <t>Trung bình</t>
+  </si>
+  <si>
+    <t>Trùng D1 khu trục</t>
+  </si>
+  <si>
+    <t>Thấp</t>
+  </si>
+  <si>
+    <t>85 km/h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1000 km/h </t>
+  </si>
+  <si>
+    <t>ss</t>
+  </si>
+  <si>
+    <t>115 km/h</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -259,11 +280,37 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -274,7 +321,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -349,11 +396,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -365,13 +421,19 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -654,7 +716,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -828,13 +890,13 @@
         <v>12</v>
       </c>
       <c r="B9" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9" s="1">
         <v>4</v>
       </c>
       <c r="D9" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E9" s="1">
         <v>260</v>
@@ -879,7 +941,7 @@
         <v>14</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>25</v>
@@ -896,7 +958,7 @@
         <v>15</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>23</v>
@@ -959,7 +1021,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
@@ -970,13 +1032,13 @@
         <v>3000</v>
       </c>
       <c r="D17" s="1">
-        <v>20</v>
+        <v>200</v>
       </c>
       <c r="E17" s="1">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
@@ -993,7 +1055,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
@@ -1010,7 +1072,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>5</v>
       </c>
@@ -1027,7 +1089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>6</v>
       </c>
@@ -1044,7 +1106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>7</v>
       </c>
@@ -1061,7 +1123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>8</v>
       </c>
@@ -1078,7 +1140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>9</v>
       </c>
@@ -1095,213 +1157,238 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="29" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="29" spans="1:10" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="C29" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="D29" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E29" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="F29" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="G29" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="F29" s="3" t="s">
+      <c r="H29" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G29" s="3" t="s">
+      <c r="I29" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H29" s="3" t="s">
+      <c r="B30" s="5" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
+      <c r="C30" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B30" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="D30" s="5" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>38</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E31" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="F31" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C31" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D31" s="5" t="s">
+      <c r="G31" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E31" s="5" t="s">
+      <c r="H31" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="F31" s="5" t="s">
+      <c r="I31" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C32" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G31" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="H31" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="4" t="s">
+      <c r="D32" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F32" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B32" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E32" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="H32" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G32" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="I32" s="8"/>
+      <c r="J32" s="9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>6</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D33" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="H33" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E33" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="H33" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I33" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B34" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C35" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C34" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E34" s="5" t="s">
+      <c r="D35" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="H35" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="F34" s="5" t="s">
+      <c r="B36" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="G34" s="5" t="s">
+      <c r="C36" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="H34" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B35" s="7" t="s">
+      <c r="D36" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F36" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="G36" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D35" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="E35" s="7" t="s">
+      <c r="H36" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="F35" s="7" t="s">
+      <c r="I36" s="5" t="s">
         <v>64</v>
-      </c>
-      <c r="G35" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="H35" s="7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="G36" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="H36" s="5" t="s">
-        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>